<commit_message>
Dynamic keyword matching from Excel
</commit_message>
<xml_diff>
--- a/germany_processes.xlsx
+++ b/germany_processes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30117"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cisco-my.sharepoint.com/personal/arsreeku_cisco_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arsreeku/Desktop/germany-process-navigator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{247E14CD-E166-43D3-B4F7-0D847B1A6059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC2C709D-6700-4547-9F6D-0AC09CF4E5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="16620" xr2:uid="{F5260CA3-5578-0C4B-8595-350C47575DD7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>Process</t>
   </si>
@@ -47,155 +47,208 @@
     <t>Work hours (parttime/fulltime)</t>
   </si>
   <si>
-    <t>Region Based Part-Time Process
- Part-Time Work – Austria, Germany, Ireland, Netherlands &amp; UK
-For employees in Austria, Germany, Ireland, Netherlands &amp; UK: Please make sure the HR Service is ‘Employee Data Change
-Request’ and re-assign the case to Country Team selecting ‘HRSD_Country_Support_EMEA’ Assignment Group.
-Country Team ensures the contract addendum is signed and sent a task to Transactions Team for data entry.
-➢ Country Team sends a task to ETP team with details, employee name &amp; ID, Effective Date of change, Work hours per week &amp;
-Work Schedule
-➢ ETP Team to check the availability of work schedule before proceeding with work hours change update in Workday.
-➢ ETP team completes the Workday Update as per the process steps.
-➢ Once the work hours change is submitted, the transaction is routed for 1st &amp; 2nd level manager approvals. Notify country
-support that the work hours change has been submitted and is pending manager approvals.
-➢ On completion of approvals in Workday, submit work schedule and notify country support and Close the task.
-Note 1-Germany: If a case to change the working hours is opened for an Intern, the request form and contract addendum
-are not required. The case requester must provide the manager’s approval for the change confirming the impacted intern’s
-name, the effective date of the change, new weekly working hours, and new working schedule. Once the approvals are
-provided, ETP enters new working hours in Workday and assign the work schedule.</t>
-  </si>
-  <si>
     <t>Personal Data</t>
   </si>
   <si>
-    <t xml:space="preserve">Citizenship change:  
-Document required: ID Proof issued by Government 
-Process Steps:  
-Verify the attached documents  
-Approve/Send back the transaction 
-For Germany Citizenship update, before approving the tasks, Download &amp; Pfile the Passport/ID Proof </t>
-  </si>
-  <si>
     <t>Job Title</t>
   </si>
   <si>
-    <t>Germany: Ensure the HR service is marked as 'Lateral Job Change.' Reassign the case to the Country Team by selecting the ' HRSD_Country_Support_EMEA'' assignment group. The Country Team will handle signing the contract addendum and will send a task to the Transactions Team for data entry for the Workday updates within scope of ETP Team. WC approval needed</t>
-  </si>
-  <si>
     <t>NYR/MYR</t>
   </si>
   <si>
-    <t>Germany-Specific Cases: • Transferred all cases for employees in Germany to country support team for Works Council approval &amp; addendum preparation. Country Support team will set Task for workday updated when both are in place.</t>
-  </si>
-  <si>
     <t>Sup org changes</t>
   </si>
   <si>
-    <t>For changes for employees in Germany: Moving Worker(s) across Supervisory Organizations in
-Germany requires completion and submission of this additional form which will be provided to the
-Workers Council.
-► Rep to set a task to Germany Country Support Team for Worker Council approval, by sending a task to HRSD_Country_Support_EMEA.
-Once approval is received from CS, TS to process with data entry</t>
-  </si>
-  <si>
     <t>Internship extension</t>
   </si>
   <si>
-    <t>Germany Please make sure the HR Service is ‘Employee Data Change Request’ and re-assign the case to Country Team selecting ‘HRSD_Country_Support’ Assignment Group. Country Team ensures the contract addendum is signed and sent a task to Transactions Team for data entry.</t>
-  </si>
-  <si>
     <t>Voluntary Termination</t>
   </si>
   <si>
-    <t xml:space="preserve">In Germany, exit date must be either on the 15th or the last day of the month. 
-The Regrettable and Eligible for Rehire fields must always be Yes for Employees in Austria, Belgium, France, Germany, or the Netherlands. </t>
-  </si>
-  <si>
     <t>Work Location</t>
   </si>
   <si>
-    <t>In Austria, Switzerland, Germany, France, Italy, Spain, Portugal and Egypt employees do not
-have an offsite Work Space.
+    <t>Hybrid work policy</t>
+  </si>
+  <si>
+    <t>Global Start Date corrections</t>
+  </si>
+  <si>
+    <t>EMEA PTO Carryover</t>
+  </si>
+  <si>
+    <t>Germany Sick Time</t>
+  </si>
+  <si>
+    <t>Modifying Talent Assessments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only active regular and fixed term employees (except for employees with work country of Austria, France, Germany, Netherlands) on 5/9 will have talent assessments in Workday. Only the leader as of 5/9 will receive a talent assessment (for employees who move, it is the responsibility of the prior leader to complete). </t>
+  </si>
+  <si>
+    <t>Employee Type change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dual Students (Germany): To transition to a permanent role, a new requisition must be created. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leitender Mitarbeiter Status </t>
+  </si>
+  <si>
+    <t>In Germany, the status of Leitender Mitarbeiter is not tied to a specific job role but applies to employees who are part of the leadership team or have managerial responsibility. This may include individuals in positions responsible for managing teams or key business functions.
+For any related process, they get a special addendum of the status of "Leitender Mitarbeiter". Also the standard CS process should be followed first. A review will then determine whether additional approval (e.g., WC approval) is required or if only the  addendum needs to be applied</t>
+  </si>
+  <si>
+    <t>Process:
+1) Please make sure the HR Service is ‘Employee Data Change Request’ and re-assign the case to CS selecting ‘HRSD_Country_Support_EMEA’ Assignment Group.
+2) CS Team ensures the contract addendum is signed and sends a task to TS for data entry.
+3) The task to TS team should contain details, employee name &amp; ID, Effective Date of change, Work hours per week &amp; Work Schedule
+4) TS  to check the availability of work schedule before proceeding with work hours change update in Workday.
+5) TS completes the Workday Update as per the process steps.
+6) Once the work hours change is submitted, the transaction is routed for 1st &amp; 2nd level manager approvals. TS to notify CS that the work hours change has been submitted and is pending manager approvals.
+7) On completion of approvals in Workday, TS to submit work schedule and notify CS and Close the task.
+Special Considerations: 
+1) If a case to change the working hours is opened for an Intern, the request form and contract addendumare not required. 
+2) The case requester must provide the manager’s approval for the change confirming the impacted intern’s name, the effective date of the change, new weekly working hours, and new working schedule. 
+3) Once the approvals are provided, TS enters new working hours in Workday and assign the work schedule.</t>
+  </si>
+  <si>
+    <t>Process: 
+1) TS to Ensure the HR service is marked as 'Lateral Job Change' &amp; Reassign the case to the CS by selecting the ' HRSD_Country_Support_EMEA'' assignment group. 
+2) CS will handle signing the contract addendum and will send a task to the Transactions Team for data entry for the Workday updates within scope of ETP Team. 
+Special Considerations: WC approval needed</t>
+  </si>
+  <si>
+    <t>Process: 
+1) TS to transfer all cases for employees in Germany to CS team for Works Council approval &amp; addendum preparation. 
+2) CS team will set Task for workday updated when both are in place.</t>
+  </si>
+  <si>
+    <t>Process:
+1) For changes for employees in Germany: Moving Worker(s) across Supervisory Organizations in Germany requires completion and submission of this additional form which will be provided to the Workers Council.
+2) TS to set a task to CS Team for Worker Council approval, by sending a task to HRSD_Country_Support_EMEA.
+3) Once approval is received from CS, TS to process with data entry
+Special Considerations: WC approval needed</t>
+  </si>
+  <si>
+    <t>Process: 
+1) TS to make sure the HR Service is ‘Employee Data Change Request’ and re-assign the case to CS Team by selecting ‘HRSD_Country_Support’ Assignment Group. 
+2) CS Team ensures the contract addendum is signed and sent a task to TS Team for data entry.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Process: 
+1) In Germany, exit date must be either on the 15th or the last day of the month. 
+2) The Regrettable and Eligible for Rehire fields must always be Yes. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Process:
+1) For changes for employees in Germany: TS to make sure the HR Service is ‘Employee Data Change Request’ and re-assign the case to CS Team selecting ‘HRSD_Country_Support_EMEA’ Assignment Group. 
+2) CS Team ensures the contract addendum is signed and sent and then will send a task to TS Team for data entry.
 Other Considerations:
-For changes for employees in Germany: Please make sure the HR Service is ‘Employee Data Change
-Request’ and re-assign the case to Country Team selecting ‘HRSD_Country_Support_EMEA’
-Assignment Group. Country Team ensures the contract addendum is signed and sent and then will send a
-task to Transactions Team for data entry.</t>
-  </si>
-  <si>
-    <t>Hybrid work policy</t>
-  </si>
-  <si>
-    <t>Please use this template for the following countries until further notice (France, Germany, Spain, Portugal, Belgium, Luxembourg, Kuwait, Poland, Russia CIS, Austria)
-Our previous Flexible Working policies and guidelines have recently been reviewed and our new Hybrid Working guidelines and policies have now been published.​
+Employees in Germany do not have an offsite Work Space.
+</t>
+  </si>
+  <si>
+    <t>Process:
+1) TS to convey the below: Previous Flexible Working policies and guidelines have recently been reviewed and our new Hybrid Working guidelines and policies have now been published.​
 https://cisco.sharepoint.com/sites/move-to-hybrid-world/SitePages/Hybrid-World-and-Office-Entry-FAQ.aspx#hybrid-policies-guidelines-questions​
 information is published.  We will be happy to support you. Work is now underway to determine the impact to our previous flexible working policies locally (in country). Whilst this review is being carried out any changes to remote worker status as well as new requests to become a remote worker will be put on hold.  ​
 As such, we hope you don’t mind if we now move this case to a resolved status. However please do keep an eye on the Hybrid Working SharePoint site for further updates, once they are available. ​
 Please do not hesitate to get back in touch with us once further country-specific ​</t>
   </si>
   <si>
-    <t>Global Start Date corrections</t>
-  </si>
-  <si>
-    <t>Effective Date Correction:
-The content below outlines the steps for correcting Workday transaction’s (Event) effective date, for
-instance, Promotion, Transfer, Lateral updates, or any Data Change transactions.
-Note: (For Germany)- Rep to set a task to CS and check if a new addendum needs to be issued &amp; approval from WC is required</t>
-  </si>
-  <si>
-    <t>EMEA PTO Carryover</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Germany: 
-Cases with a request to move above 10 days of PTO should be re-assigned to Country Team to HRSD_Country _Support EMEA. 
-Cases with a request to extend carry over after 31st March 2025 should be re-assigned to Country Team HRSD_Country _Support EMEA. 
-Cases with a request to move PTO days up to 10 days but not beyond 31st March should be handled by us. In such scenario we need to inform the employee that carry over will be done automatically by the system and carried over days will expire on 1st April 2025. </t>
-  </si>
-  <si>
-    <t>Germany Sick Time</t>
-  </si>
-  <si>
-    <t>Process Guide</t>
-  </si>
-  <si>
-    <t>Modifying Talent Assessments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only active regular and fixed term employees (except for employees with work country of Austria, France, Germany, Netherlands) on 5/9 will have talent assessments in Workday. Only the leader as of 5/9 will receive a talent assessment (for employees who move, it is the responsibility of the prior leader to complete). </t>
-  </si>
-  <si>
-    <t>Employee Type change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dual Students (Germany): To transition to a permanent role, a new requisition must be created. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leitender Mitarbeiter Status </t>
-  </si>
-  <si>
-    <t>In Germany, the status of Leitender Mitarbeiter is not tied to a specific job role but applies to employees who are part of the leadership team or have managerial responsibility. This may include individuals in positions responsible for managing teams or key business functions.
-For any related process, they get a special addendum of the status of "Leitender Mitarbeiter". Also the standard CS process should be followed first. A review will then determine whether additional approval (e.g., WC approval) is required or if only the  addendum needs to be applied</t>
-  </si>
-  <si>
-    <t>what about LOA requests</t>
+    <t>For Germany Effective Date Correction (correcting Workday transaction’s effective date, for instance, Promotion, Transfer, Lateral updates, or any Data Change transactions) : TS Rep to set a task to CS and check if a new addendum needs to be issued &amp; approval from WC is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Process:
+1) Cases with a request to move above 10 days of PTO should be re-assigned by TS to CS Team to HRSD_Country _Support EMEA. 
+2) Cases with a request to extend carry over after 31st March 2025 should be re-assigned by TS to CS Team HRSD_Country _Support EMEA. 
+3) Cases with a request to move PTO days up to 10 days but not beyond 31st March should be handled by TS. In such scenario TS should inform the employee that carry over will be done automatically by the system and carried over days will expire on 1st April 2025. </t>
+  </si>
+  <si>
+    <t>Key points:
+• CS Team approval is required for new entries, corrections, and cancellations via SNOW.
+• Sick Time (No Sick Note) does not require Country Team approval.
+• Entries/corrections beyond 90 days additionally require Workday Team approval.
+Leave types:
+• Sick Time (No Sick Note): for calendar days 1–2 only.
+• Sick Time (With Sick Note): for calendar days 3–42, or from day 1 if certified earlier. Upload rules differ for private vs statutory insurance.
+• Medical Leave (Krankengeld): applicable from day 43 onwards for the same illness.
+Additional notes:
+• If the sick note includes weekends/public holidays, those days must also be recorded in Workday.
+• Corrections must align with the doctor’s certificate; early return requires a health note.
+• For statutory insured employees, corrected sick notes do not need to be shared with the employer, but must still be issued.
+Cancellation/correction scenarios supported:
+• Partial cancellation of Sick Time (With Sick Note)
+• Full cancellation of Sick Time (With Sick Note)
+• Full cancellation of Sick Time (No Sick Note)
+• Partial cancellation of Sick Time (No Sick Note)
+In all correction/cancellation cases, ensure the case number is added in the “Comment” and “Comment to Approver” fields.</t>
+  </si>
+  <si>
+    <t>Keywords</t>
+  </si>
+  <si>
+    <t>workhours, work hours, WORK HOURS, WORKHOURS, Workhours, parttime, fulltime, part time, full time, working schedule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Process for updating Citizenship: 
+1) TS to Request for ID Proof issued by Government 
+2) Verify the attached documents  
+3) Approve/Send back the transaction 
+Special Considerations: For Germany Citizenship update, before approving the tasks, Download &amp; Pfile the Passport/ID Proof </t>
+  </si>
+  <si>
+    <t>Citizenship, citizen, update citizen</t>
+  </si>
+  <si>
+    <t>job title, jobtitle, Job Title, Jobtitle, Job change, JOB Changes</t>
+  </si>
+  <si>
+    <t>NYR, MYR, NYR/MYR, New year rediness</t>
+  </si>
+  <si>
+    <t>Sup Org changes, manager changes, changing manager, update manager, new manager</t>
+  </si>
+  <si>
+    <t>extend intern, internship extension, internship, extension of internship</t>
+  </si>
+  <si>
+    <t>termination, last day, regrettable, rehire</t>
+  </si>
+  <si>
+    <t>location, work location, work space</t>
+  </si>
+  <si>
+    <t>hybrid, WFH</t>
+  </si>
+  <si>
+    <t>effective date, start date</t>
+  </si>
+  <si>
+    <t>PTO</t>
+  </si>
+  <si>
+    <t>Sick time, sick day, sick noye</t>
+  </si>
+  <si>
+    <t>talent assessment, TA</t>
+  </si>
+  <si>
+    <t>EMPLOYEE TYPE,DUAL STUDENTS, PERMANENT</t>
+  </si>
+  <si>
+    <t>Leitender Mitarbeiter Status , LEADERSHIP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -232,11 +285,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -247,18 +299,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -591,151 +639,194 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50947E45-34EF-2847-8AD9-576C705E0B0C}">
-  <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.95"/>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="104.375" style="2" customWidth="1"/>
-    <col min="3" max="16384" width="10.875" style="2"/>
+    <col min="2" max="2" width="104.33203125" style="2" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="365.25" customHeight="1">
+      <c r="C1" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="365.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="221.1">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="75" customHeight="1">
-      <c r="A4" s="2" t="s">
+      <c r="B5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="119" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="68" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="51">
-      <c r="A5" s="2" t="s">
+      <c r="B7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="136" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="102">
-      <c r="A6" s="2" t="s">
+      <c r="B9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="187" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="51">
-      <c r="A7" s="2" t="s">
+      <c r="B11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="136" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B12" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="388" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="68.099999999999994">
-      <c r="A8" s="2" t="s">
+      <c r="B13" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B14" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="135.94999999999999">
-      <c r="A9" s="2" t="s">
+      <c r="C14" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="288.95">
-      <c r="A10" s="2" t="s">
+      <c r="C15" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="119" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="84.95">
-      <c r="A11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="186.95">
-      <c r="A12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="51">
-      <c r="A14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="119.1">
-      <c r="A16" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1">
-      <c r="A18" s="6" t="s">
-        <v>32</v>
-      </c>
+      <c r="C16" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="5"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B13" r:id="rId1" xr:uid="{E189E44F-8CF7-B449-BFDA-98FCCD201644}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddFooter>&amp;R_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Cisco Confidential</oddFooter>

</xml_diff>